<commit_message>
calibration figures; update fft
</commit_message>
<xml_diff>
--- a/table2_all_models.xlsx
+++ b/table2_all_models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\27261\Desktop\3_Courses in PHBS\3_09_AppliedStochasticProcess\Project_sv32_EMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E316565C-5450-41BE-A709-C124D0A99B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89E18294-EA77-41DC-9EB7-E7F5C2BD1BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -334,36 +334,28 @@
     <t>0.0009893 (0.01%)</t>
   </si>
   <si>
-    <t>8.197e+58 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1.314e+59 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1.624e+59 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1.772e+59 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1.784e+59 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>6.397e+59 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>-2.655e+58 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>-5.957e+59 (nan%)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <t>0.0003048 (0.00%)</t>
+  </si>
+  <si>
+    <t>0.068 (1.05%)</t>
+  </si>
+  <si>
+    <t>0.001088 (0.02%)</t>
+  </si>
+  <si>
+    <t>0.001157 (0.02%)</t>
+  </si>
+  <si>
+    <t>0.001138 (0.02%)</t>
+  </si>
+  <si>
+    <t>0.0015 (0.00%)</t>
+  </si>
+  <si>
+    <t>0.001557 (0.01%)</t>
+  </si>
+  <si>
+    <t>0.002021 (0.02%)</t>
   </si>
 </sst>
 </file>
@@ -465,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -473,17 +465,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -807,34 +798,34 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="6"/>
+      <c r="E1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="3" t="s">
+      <c r="F1" s="6"/>
+      <c r="G1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="4"/>
-      <c r="I1" s="3" t="s">
+      <c r="H1" s="6"/>
+      <c r="I1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="4"/>
-      <c r="K1" s="3" t="s">
+      <c r="J1" s="6"/>
+      <c r="K1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="3" t="s">
+      <c r="L1" s="6"/>
+      <c r="M1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="3" t="s">
+      <c r="N1" s="6"/>
+      <c r="O1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="4"/>
+      <c r="P1" s="6"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -927,864 +918,903 @@
         <v>16</v>
       </c>
       <c r="M4" s="2">
-        <v>6.8426199955865741E-2</v>
+        <v>0.34941570018418128</v>
       </c>
       <c r="N4" t="s">
         <v>17</v>
       </c>
       <c r="O4" s="2">
-        <v>0.51162280002608895</v>
+        <v>0.21686759986914689</v>
       </c>
       <c r="P4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="1">
         <v>95</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="3">
         <v>95.302338999928907</v>
       </c>
       <c r="D5" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="3">
         <v>13.48963779991027</v>
       </c>
       <c r="F5" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="3">
         <v>4.8519699950702488E-2</v>
       </c>
       <c r="H5" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="3">
         <v>0.33104970003478229</v>
       </c>
       <c r="J5" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="3">
         <v>0.32904240000061691</v>
       </c>
       <c r="L5" t="s">
         <v>22</v>
       </c>
-      <c r="M5" s="7">
-        <v>6.9130799965932965E-2</v>
+      <c r="M5" s="3">
+        <v>0.18376509984955189</v>
       </c>
       <c r="N5" t="s">
         <v>23</v>
       </c>
-      <c r="O5" s="7">
-        <v>0.19818639999721199</v>
+      <c r="O5" s="3">
+        <v>0.1025725000072271</v>
       </c>
       <c r="P5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
+      <c r="A6" s="7"/>
       <c r="B6" s="1">
         <v>100</v>
       </c>
-      <c r="C6" s="8"/>
+      <c r="C6" s="4"/>
       <c r="D6" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="8"/>
+      <c r="E6" s="4"/>
       <c r="F6" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="8"/>
+      <c r="G6" s="4"/>
       <c r="H6" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="8"/>
+      <c r="I6" s="4"/>
       <c r="J6" t="s">
         <v>25</v>
       </c>
-      <c r="K6" s="8"/>
+      <c r="K6" s="4"/>
       <c r="L6" t="s">
         <v>26</v>
       </c>
-      <c r="M6" s="8"/>
+      <c r="M6" s="4"/>
       <c r="N6" t="s">
         <v>27</v>
       </c>
-      <c r="O6" s="8"/>
+      <c r="O6" s="4"/>
       <c r="P6" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A7" s="6"/>
+      <c r="A7" s="8"/>
       <c r="B7" s="1">
         <v>105</v>
       </c>
-      <c r="C7" s="8"/>
+      <c r="C7" s="4"/>
       <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="8"/>
+      <c r="E7" s="4"/>
       <c r="F7" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="8"/>
+      <c r="G7" s="4"/>
       <c r="H7" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="8"/>
+      <c r="I7" s="4"/>
       <c r="J7" t="s">
         <v>29</v>
       </c>
-      <c r="K7" s="8"/>
+      <c r="K7" s="4"/>
       <c r="L7" t="s">
         <v>30</v>
       </c>
-      <c r="M7" s="8"/>
+      <c r="M7" s="4"/>
       <c r="N7" t="s">
         <v>31</v>
       </c>
-      <c r="O7" s="8"/>
+      <c r="O7" s="4"/>
       <c r="P7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B8" s="1">
         <v>95</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="3">
         <v>70.396328600007109</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="3">
         <v>9.5038490999722853</v>
       </c>
       <c r="F8" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="3">
         <v>4.3361600022763007E-2</v>
       </c>
       <c r="H8" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="3">
         <v>0.34853079996537423</v>
       </c>
       <c r="J8" t="s">
         <v>34</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="3">
         <v>0.3853117999387905</v>
       </c>
       <c r="L8" t="s">
         <v>35</v>
       </c>
-      <c r="M8" s="7">
-        <v>6.4975899993441999E-2</v>
+      <c r="M8" s="3">
+        <v>0.26901280018500978</v>
       </c>
       <c r="N8" t="s">
         <v>36</v>
       </c>
-      <c r="O8" s="7">
-        <v>0.25475169997662311</v>
+      <c r="O8" s="3">
+        <v>0.13974429992958901</v>
       </c>
       <c r="P8" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
+      <c r="A9" s="7"/>
       <c r="B9" s="1">
         <v>100</v>
       </c>
-      <c r="C9" s="8"/>
+      <c r="C9" s="4"/>
       <c r="D9" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="8"/>
+      <c r="E9" s="4"/>
       <c r="F9" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="8"/>
+      <c r="G9" s="4"/>
       <c r="H9" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="8"/>
+      <c r="I9" s="4"/>
       <c r="J9" t="s">
         <v>38</v>
       </c>
-      <c r="K9" s="8"/>
+      <c r="K9" s="4"/>
       <c r="L9" t="s">
         <v>39</v>
       </c>
-      <c r="M9" s="8"/>
+      <c r="M9" s="4"/>
       <c r="N9" t="s">
         <v>40</v>
       </c>
-      <c r="O9" s="8"/>
+      <c r="O9" s="4"/>
       <c r="P9" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
+      <c r="A10" s="8"/>
       <c r="B10" s="1">
         <v>105</v>
       </c>
-      <c r="C10" s="8"/>
+      <c r="C10" s="4"/>
       <c r="D10" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="8"/>
+      <c r="E10" s="4"/>
       <c r="F10" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="8"/>
+      <c r="G10" s="4"/>
       <c r="H10" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="8"/>
+      <c r="I10" s="4"/>
       <c r="J10" t="s">
         <v>42</v>
       </c>
-      <c r="K10" s="8"/>
+      <c r="K10" s="4"/>
       <c r="L10" t="s">
         <v>43</v>
       </c>
-      <c r="M10" s="8"/>
+      <c r="M10" s="4"/>
       <c r="N10" t="s">
         <v>44</v>
       </c>
-      <c r="O10" s="8"/>
+      <c r="O10" s="4"/>
       <c r="P10" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B11" s="1">
         <v>47</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="3">
         <v>99.31938280002214</v>
       </c>
       <c r="D11" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="3">
         <v>8.9469167999923229</v>
       </c>
       <c r="F11" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="3">
         <v>3.3504700055345893E-2</v>
       </c>
       <c r="H11" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="3">
         <v>24.67282950005028</v>
       </c>
       <c r="J11" t="s">
         <v>47</v>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="3">
         <v>24.9390296000056</v>
       </c>
       <c r="L11" t="s">
         <v>48</v>
       </c>
-      <c r="M11" s="7">
-        <v>6.7150399903766811E-2</v>
+      <c r="M11" s="3">
+        <v>14.420765599934381</v>
       </c>
       <c r="N11" t="s">
         <v>104</v>
       </c>
-      <c r="O11" s="7">
-        <v>14.10810660000425</v>
+      <c r="O11" s="3">
+        <v>6.9287210998591036</v>
       </c>
       <c r="P11" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
+      <c r="A12" s="7"/>
       <c r="B12" s="1">
         <v>48</v>
       </c>
-      <c r="C12" s="8"/>
+      <c r="C12" s="4"/>
       <c r="D12" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="4"/>
       <c r="F12" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="8"/>
+      <c r="G12" s="4"/>
       <c r="H12" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="8"/>
+      <c r="I12" s="4"/>
       <c r="J12" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="8"/>
+      <c r="K12" s="4"/>
       <c r="L12" t="s">
         <v>51</v>
       </c>
-      <c r="M12" s="8"/>
+      <c r="M12" s="4"/>
       <c r="N12" t="s">
         <v>105</v>
       </c>
-      <c r="O12" s="8"/>
+      <c r="O12" s="4"/>
       <c r="P12" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
+      <c r="A13" s="7"/>
       <c r="B13" s="1">
         <v>49</v>
       </c>
-      <c r="C13" s="8"/>
+      <c r="C13" s="4"/>
       <c r="D13" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="4"/>
       <c r="F13" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="8"/>
+      <c r="G13" s="4"/>
       <c r="H13" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="8"/>
+      <c r="I13" s="4"/>
       <c r="J13" t="s">
         <v>53</v>
       </c>
-      <c r="K13" s="8"/>
+      <c r="K13" s="4"/>
       <c r="L13" t="s">
         <v>54</v>
       </c>
-      <c r="M13" s="8"/>
+      <c r="M13" s="4"/>
       <c r="N13" t="s">
         <v>106</v>
       </c>
-      <c r="O13" s="8"/>
+      <c r="O13" s="4"/>
       <c r="P13" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
+      <c r="A14" s="7"/>
       <c r="B14" s="1">
         <v>50</v>
       </c>
-      <c r="C14" s="8"/>
+      <c r="C14" s="4"/>
       <c r="D14" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="8"/>
+      <c r="E14" s="4"/>
       <c r="F14" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="8"/>
+      <c r="G14" s="4"/>
       <c r="H14" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="8"/>
+      <c r="I14" s="4"/>
       <c r="J14" t="s">
         <v>56</v>
       </c>
-      <c r="K14" s="8"/>
+      <c r="K14" s="4"/>
       <c r="L14" t="s">
         <v>57</v>
       </c>
-      <c r="M14" s="8"/>
+      <c r="M14" s="4"/>
       <c r="N14" t="s">
         <v>107</v>
       </c>
-      <c r="O14" s="8"/>
+      <c r="O14" s="4"/>
       <c r="P14" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
+      <c r="A15" s="8"/>
       <c r="B15" s="1">
         <v>51</v>
       </c>
-      <c r="C15" s="8"/>
+      <c r="C15" s="4"/>
       <c r="D15" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="8"/>
+      <c r="E15" s="4"/>
       <c r="F15" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="8"/>
+      <c r="G15" s="4"/>
       <c r="H15" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="8"/>
+      <c r="I15" s="4"/>
       <c r="J15" t="s">
         <v>59</v>
       </c>
-      <c r="K15" s="8"/>
+      <c r="K15" s="4"/>
       <c r="L15" t="s">
         <v>60</v>
       </c>
-      <c r="M15" s="8"/>
+      <c r="M15" s="4"/>
       <c r="N15" t="s">
         <v>108</v>
       </c>
-      <c r="O15" s="8"/>
+      <c r="O15" s="4"/>
       <c r="P15" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="5" t="s">
         <v>62</v>
       </c>
       <c r="B16" s="1">
         <v>10</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="3">
         <v>110.7483931999886</v>
       </c>
       <c r="D16" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="3">
         <v>8.7633946998976171</v>
       </c>
       <c r="F16" t="s">
         <v>20</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="3">
         <v>3.2180099980905652E-2</v>
       </c>
       <c r="H16" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="3">
         <v>25.133232499938462</v>
       </c>
       <c r="J16" t="s">
         <v>63</v>
       </c>
-      <c r="K16" s="7">
+      <c r="K16" s="3">
         <v>24.05367499997374</v>
       </c>
       <c r="L16" t="s">
         <v>64</v>
       </c>
-      <c r="M16" s="7">
-        <v>6.8539600004442036E-2</v>
+      <c r="M16" s="3">
+        <v>14.51756930002011</v>
       </c>
       <c r="N16" t="s">
         <v>109</v>
       </c>
-      <c r="O16" s="7">
-        <v>11.94073160004336</v>
+      <c r="O16" s="3">
+        <v>6.8659487999975681</v>
       </c>
       <c r="P16" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
+      <c r="A17" s="7"/>
       <c r="B17" s="1">
         <v>20</v>
       </c>
-      <c r="C17" s="8"/>
+      <c r="C17" s="4"/>
       <c r="D17" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="8"/>
+      <c r="E17" s="4"/>
       <c r="F17" t="s">
         <v>20</v>
       </c>
-      <c r="G17" s="8"/>
+      <c r="G17" s="4"/>
       <c r="H17" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="8"/>
+      <c r="I17" s="4"/>
       <c r="J17" t="s">
         <v>66</v>
       </c>
-      <c r="K17" s="8"/>
+      <c r="K17" s="4"/>
       <c r="L17" t="s">
         <v>67</v>
       </c>
-      <c r="M17" s="8"/>
-      <c r="N17" s="9" t="s">
+      <c r="M17" s="4"/>
+      <c r="N17" t="s">
         <v>110</v>
       </c>
-      <c r="O17" s="8"/>
+      <c r="O17" s="4"/>
       <c r="P17" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A18" s="6"/>
+      <c r="A18" s="8"/>
       <c r="B18" s="1">
         <v>40</v>
       </c>
-      <c r="C18" s="8"/>
+      <c r="C18" s="4"/>
       <c r="D18" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="4"/>
       <c r="F18" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="8"/>
+      <c r="G18" s="4"/>
       <c r="H18" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="8"/>
+      <c r="I18" s="4"/>
       <c r="J18" t="s">
         <v>69</v>
       </c>
-      <c r="K18" s="8"/>
+      <c r="K18" s="4"/>
       <c r="L18" t="s">
         <v>70</v>
       </c>
-      <c r="M18" s="8"/>
-      <c r="N18" s="9" t="s">
+      <c r="M18" s="4"/>
+      <c r="N18" t="s">
         <v>111</v>
       </c>
-      <c r="O18" s="8"/>
+      <c r="O18" s="4"/>
       <c r="P18" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="5" t="s">
         <v>72</v>
       </c>
       <c r="B19" s="1">
         <v>47</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="3">
         <v>104.217961300048</v>
       </c>
       <c r="D19" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="3">
         <v>34.606527099967927</v>
       </c>
       <c r="F19" t="s">
         <v>20</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="3">
         <v>5.8478599996306002E-2</v>
       </c>
       <c r="H19" t="s">
         <v>20</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="3">
         <v>0.33090339996851981</v>
       </c>
       <c r="J19" t="s">
         <v>73</v>
       </c>
-      <c r="K19" s="7">
+      <c r="K19" s="3">
         <v>0.35076990001834929</v>
       </c>
       <c r="L19" t="s">
         <v>74</v>
       </c>
-      <c r="M19" s="7">
-        <v>6.4650999964214861E-2</v>
+      <c r="M19" s="3">
+        <v>0.20381490001454949</v>
       </c>
       <c r="N19" t="s">
         <v>75</v>
       </c>
-      <c r="O19" s="7">
-        <v>0.1574922000290826</v>
+      <c r="O19" s="3">
+        <v>8.7652200134471059E-2</v>
       </c>
       <c r="P19" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
+      <c r="A20" s="7"/>
       <c r="B20" s="1">
         <v>48</v>
       </c>
-      <c r="C20" s="8"/>
+      <c r="C20" s="4"/>
       <c r="D20" t="s">
         <v>20</v>
       </c>
-      <c r="E20" s="8"/>
+      <c r="E20" s="4"/>
       <c r="F20" t="s">
         <v>20</v>
       </c>
-      <c r="G20" s="8"/>
+      <c r="G20" s="4"/>
       <c r="H20" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="8"/>
+      <c r="I20" s="4"/>
       <c r="J20" t="s">
         <v>77</v>
       </c>
-      <c r="K20" s="8"/>
+      <c r="K20" s="4"/>
       <c r="L20" t="s">
         <v>78</v>
       </c>
-      <c r="M20" s="8"/>
+      <c r="M20" s="4"/>
       <c r="N20" t="s">
         <v>79</v>
       </c>
-      <c r="O20" s="8"/>
+      <c r="O20" s="4"/>
       <c r="P20" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
+      <c r="A21" s="7"/>
       <c r="B21" s="1">
         <v>49</v>
       </c>
-      <c r="C21" s="8"/>
+      <c r="C21" s="4"/>
       <c r="D21" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="8"/>
+      <c r="E21" s="4"/>
       <c r="F21" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="8"/>
+      <c r="G21" s="4"/>
       <c r="H21" t="s">
         <v>20</v>
       </c>
-      <c r="I21" s="8"/>
+      <c r="I21" s="4"/>
       <c r="J21" t="s">
         <v>81</v>
       </c>
-      <c r="K21" s="8"/>
+      <c r="K21" s="4"/>
       <c r="L21" t="s">
         <v>82</v>
       </c>
-      <c r="M21" s="8"/>
+      <c r="M21" s="4"/>
       <c r="N21" t="s">
         <v>83</v>
       </c>
-      <c r="O21" s="8"/>
+      <c r="O21" s="4"/>
       <c r="P21" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
+      <c r="A22" s="7"/>
       <c r="B22" s="1">
         <v>50</v>
       </c>
-      <c r="C22" s="8"/>
+      <c r="C22" s="4"/>
       <c r="D22" t="s">
         <v>20</v>
       </c>
-      <c r="E22" s="8"/>
+      <c r="E22" s="4"/>
       <c r="F22" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="8"/>
+      <c r="G22" s="4"/>
       <c r="H22" t="s">
         <v>20</v>
       </c>
-      <c r="I22" s="8"/>
+      <c r="I22" s="4"/>
       <c r="J22" t="s">
         <v>85</v>
       </c>
-      <c r="K22" s="8"/>
+      <c r="K22" s="4"/>
       <c r="L22" t="s">
         <v>86</v>
       </c>
-      <c r="M22" s="8"/>
+      <c r="M22" s="4"/>
       <c r="N22" t="s">
         <v>87</v>
       </c>
-      <c r="O22" s="8"/>
+      <c r="O22" s="4"/>
       <c r="P22" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
+      <c r="A23" s="8"/>
       <c r="B23" s="1">
         <v>51</v>
       </c>
-      <c r="C23" s="8"/>
+      <c r="C23" s="4"/>
       <c r="D23" t="s">
         <v>20</v>
       </c>
-      <c r="E23" s="8"/>
+      <c r="E23" s="4"/>
       <c r="F23" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="8"/>
+      <c r="G23" s="4"/>
       <c r="H23" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="8"/>
+      <c r="I23" s="4"/>
       <c r="J23" t="s">
         <v>89</v>
       </c>
-      <c r="K23" s="8"/>
+      <c r="K23" s="4"/>
       <c r="L23" t="s">
         <v>90</v>
       </c>
-      <c r="M23" s="8"/>
+      <c r="M23" s="4"/>
       <c r="N23" t="s">
         <v>91</v>
       </c>
-      <c r="O23" s="8"/>
+      <c r="O23" s="4"/>
       <c r="P23" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="5" t="s">
         <v>93</v>
       </c>
       <c r="B24" s="1">
         <v>95</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="3">
         <v>107.37175049993679</v>
       </c>
       <c r="D24" t="s">
         <v>20</v>
       </c>
-      <c r="E24" s="7">
+      <c r="E24" s="3">
         <v>8.9517658000113443</v>
       </c>
       <c r="F24" t="s">
         <v>20</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="3">
         <v>5.0093900063075132E-2</v>
       </c>
       <c r="H24" t="s">
         <v>20</v>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="3">
         <v>0.34881779993884271</v>
       </c>
       <c r="J24" t="s">
         <v>34</v>
       </c>
-      <c r="K24" s="7">
+      <c r="K24" s="3">
         <v>0.33624570001848042</v>
       </c>
       <c r="L24" t="s">
         <v>35</v>
       </c>
-      <c r="M24" s="7">
-        <v>6.6565599991008639E-2</v>
+      <c r="M24" s="3">
+        <v>0.29703900008462369</v>
       </c>
       <c r="N24" t="s">
         <v>94</v>
       </c>
-      <c r="O24" s="7">
-        <v>0.25474090001080191</v>
+      <c r="O24" s="3">
+        <v>0.12931110011413691</v>
       </c>
       <c r="P24" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
+      <c r="A25" s="7"/>
       <c r="B25" s="1">
         <v>100</v>
       </c>
-      <c r="C25" s="8"/>
+      <c r="C25" s="4"/>
       <c r="D25" t="s">
         <v>20</v>
       </c>
-      <c r="E25" s="8"/>
+      <c r="E25" s="4"/>
       <c r="F25" t="s">
         <v>20</v>
       </c>
-      <c r="G25" s="8"/>
+      <c r="G25" s="4"/>
       <c r="H25" t="s">
         <v>20</v>
       </c>
-      <c r="I25" s="8"/>
+      <c r="I25" s="4"/>
       <c r="J25" t="s">
         <v>96</v>
       </c>
-      <c r="K25" s="8"/>
+      <c r="K25" s="4"/>
       <c r="L25" t="s">
         <v>97</v>
       </c>
-      <c r="M25" s="8"/>
+      <c r="M25" s="4"/>
       <c r="N25" t="s">
         <v>98</v>
       </c>
-      <c r="O25" s="8"/>
+      <c r="O25" s="4"/>
       <c r="P25" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A26" s="6"/>
+      <c r="A26" s="8"/>
       <c r="B26" s="1">
         <v>105</v>
       </c>
-      <c r="C26" s="8"/>
+      <c r="C26" s="4"/>
       <c r="D26" t="s">
         <v>20</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="4"/>
       <c r="F26" t="s">
         <v>20</v>
       </c>
-      <c r="G26" s="8"/>
+      <c r="G26" s="4"/>
       <c r="H26" t="s">
         <v>20</v>
       </c>
-      <c r="I26" s="8"/>
+      <c r="I26" s="4"/>
       <c r="J26" t="s">
         <v>100</v>
       </c>
-      <c r="K26" s="8"/>
+      <c r="K26" s="4"/>
       <c r="L26" t="s">
         <v>101</v>
       </c>
-      <c r="M26" s="8"/>
+      <c r="M26" s="4"/>
       <c r="N26" t="s">
         <v>102</v>
       </c>
-      <c r="O26" s="8"/>
+      <c r="O26" s="4"/>
       <c r="P26" t="s">
         <v>103</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="55">
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="C11:C15"/>
+    <mergeCell ref="E11:E15"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="G11:G15"/>
+    <mergeCell ref="M19:M23"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="O19:O23"/>
+    <mergeCell ref="O24:O26"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="K5:K7"/>
+    <mergeCell ref="O5:O7"/>
+    <mergeCell ref="K11:K15"/>
+    <mergeCell ref="M11:M15"/>
+    <mergeCell ref="M16:M18"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="O16:O18"/>
+    <mergeCell ref="E19:E23"/>
+    <mergeCell ref="G19:G23"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="A19:A23"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="K19:K23"/>
+    <mergeCell ref="C19:C23"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="K24:K26"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="I24:I26"/>
     <mergeCell ref="M24:M26"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="M8:M10"/>
@@ -1801,45 +1831,6 @@
     <mergeCell ref="G8:G10"/>
     <mergeCell ref="I11:I15"/>
     <mergeCell ref="M5:M7"/>
-    <mergeCell ref="A19:A23"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="K19:K23"/>
-    <mergeCell ref="C19:C23"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="K24:K26"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="I24:I26"/>
-    <mergeCell ref="M19:M23"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="O19:O23"/>
-    <mergeCell ref="O24:O26"/>
-    <mergeCell ref="A11:A15"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="K5:K7"/>
-    <mergeCell ref="O5:O7"/>
-    <mergeCell ref="K11:K15"/>
-    <mergeCell ref="M11:M15"/>
-    <mergeCell ref="M16:M18"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="O16:O18"/>
-    <mergeCell ref="E19:E23"/>
-    <mergeCell ref="G19:G23"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="I5:I7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="C11:C15"/>
-    <mergeCell ref="E11:E15"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="G5:G7"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="G11:G15"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>